<commit_message>
Update client SEO report
</commit_message>
<xml_diff>
--- a/evidence/chistograd-speed-before-after-2026-10-07.xlsx
+++ b/evidence/chistograd-speed-before-after-2026-10-07.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итоги" sheetId="1" r:id="R86c368f3fff8451c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изображения" sheetId="2" r:id="R8a291deb0cb6486d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Страницы" sheetId="3" r:id="R09f5a38f64d54de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прогоны" sheetId="4" r:id="Rc48442a0784e43e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сценарии" sheetId="5" r:id="R48b85077e8a04b26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итоги" sheetId="1" r:id="Rb54a15e0f05d48d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изображения" sheetId="2" r:id="R683f44f3a53647c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Страницы" sheetId="3" r:id="Rfcbaaaeb7dce415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прогоны" sheetId="4" r:id="Rc352bcc9c72c4d65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сценарии" sheetId="5" r:id="Rc3b4812b0c8b4274"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -537,7 +537,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Чистоград. Замеры 7 октября 2026 года.</x:v>
+        <x:v>Чистоград. Замеры 7–8 октября 2026 года (время Уфы, UTC+5).</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -616,7 +616,7 @@
       </x:c>
       <x:c r="D7" s="20" t="n">
         <x:f>'Страницы'!H7</x:f>
-        <x:v>78</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E7" s="28" t="n">
         <x:f>'Страницы'!E9</x:f>
@@ -624,7 +624,7 @@
       </x:c>
       <x:c r="F7" s="28" t="n">
         <x:f>'Страницы'!H9</x:f>
-        <x:v>3.4994288700000005</x:v>
+        <x:v>3.4032798400000006</x:v>
       </x:c>
       <x:c r="G7" s="28" t="n">
         <x:f>'Страницы'!E14/1000000</x:f>
@@ -632,7 +632,7 @@
       </x:c>
       <x:c r="H7" s="28" t="n">
         <x:f>'Страницы'!H14/1000000</x:f>
-        <x:v>1.292654</x:v>
+        <x:v>1.29283</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
@@ -648,7 +648,7 @@
       </x:c>
       <x:c r="D8" s="21" t="n">
         <x:f>'Страницы'!H20</x:f>
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E8" s="29" t="n">
         <x:f>'Страницы'!E22</x:f>
@@ -656,7 +656,7 @@
       </x:c>
       <x:c r="F8" s="29" t="n">
         <x:f>'Страницы'!H22</x:f>
-        <x:v>2.4379597800000004</x:v>
+        <x:v>2.5601073999999997</x:v>
       </x:c>
       <x:c r="G8" s="29" t="n">
         <x:f>'Страницы'!E27/1000000</x:f>
@@ -664,7 +664,7 @@
       </x:c>
       <x:c r="H8" s="29" t="n">
         <x:f>'Страницы'!H27/1000000</x:f>
-        <x:v>2.367913</x:v>
+        <x:v>2.368338</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
@@ -986,7 +986,7 @@
         <x:v>Сетевые сценарии</x:v>
       </x:c>
       <x:c r="B26" s="55" t="str">
-        <x:v>Шесть сценариев до и шесть после. По одному для каждой страницы и устройства, без замедления сети и CPU.</x:v>
+        <x:v>12 сетевых сценариев выполнены 7 октября 2026 года: шесть до и шесть после изменений.</x:v>
       </x:c>
       <x:c r="C26" s="3"/>
       <x:c r="D26" s="3"/>
@@ -998,7 +998,7 @@
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="17"/>
       <x:c r="B27" s="52" t="str">
-        <x:v>Начальная загрузка: 10 секунд после DOMContentLoaded. После прокрутки: 5 секунд. Фото: 5 секунд после</x:v>
+        <x:v>Сеть и CPU без замедления. Окна: 10 с после DOMContentLoaded, 5 с после прокрутки и открытия фото.</x:v>
       </x:c>
       <x:c r="C27" s="17"/>
       <x:c r="D27" s="17"/>
@@ -1010,7 +1010,7 @@
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="3"/>
       <x:c r="B28" s="55" t="str">
-        <x:v>открытия. Видео: 20 секунд после попытки запуска.</x:v>
+        <x:v>Видео: 20 с после попытки запуска. Шесть повторных замеров Lighthouse главной выполнены 8 октября.</x:v>
       </x:c>
       <x:c r="C28" s="3"/>
       <x:c r="D28" s="3"/>
@@ -1254,7 +1254,7 @@
         <x:v>Конец замеров, UTC</x:v>
       </x:c>
       <x:c r="B47" s="59" t="n">
-        <x:v>46302.77618642361</x:v>
+        <x:v>46302.84646997685</x:v>
       </x:c>
       <x:c r="C47" s="17"/>
       <x:c r="D47" s="17"/>
@@ -8570,11 +8570,11 @@
       </x:c>
       <x:c r="H7" s="35" t="n">
         <x:f>MEDIAN('Прогоны'!F25:F27)</x:f>
-        <x:v>78</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="I7" s="35" t="n">
         <x:f>MIN('Прогоны'!F25:F27)</x:f>
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="J7" s="35" t="n">
         <x:f>MAX('Прогоны'!F25:F27)</x:f>
@@ -8582,11 +8582,11 @@
       </x:c>
       <x:c r="K7" s="35" t="n">
         <x:f>H7-E7</x:f>
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="L7" s="42" t="n">
         <x:f>IF(E7=0,"",K7/E7)</x:f>
-        <x:v>0.7333333333333333</x:v>
+        <x:v>0.7555555555555555</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="43" customHeight="1">
@@ -8616,23 +8616,23 @@
       </x:c>
       <x:c r="H8" s="29" t="n">
         <x:f>MEDIAN('Прогоны'!G25:G27)</x:f>
-        <x:v>3.4758397099999994</x:v>
+        <x:v>3.4032798400000006</x:v>
       </x:c>
       <x:c r="I8" s="29" t="n">
         <x:f>MIN('Прогоны'!G25:G27)</x:f>
-        <x:v>3.3789251</x:v>
+        <x:v>3.3994437</x:v>
       </x:c>
       <x:c r="J8" s="29" t="n">
         <x:f>MAX('Прогоны'!G25:G27)</x:f>
-        <x:v>3.49942887</x:v>
+        <x:v>3.6228520200000003</x:v>
       </x:c>
       <x:c r="K8" s="29" t="n">
         <x:f>H8-E8</x:f>
-        <x:v>-1.3476898900000012</x:v>
+        <x:v>-1.42024976</x:v>
       </x:c>
       <x:c r="L8" s="43" t="n">
         <x:f>IF(E8=0,"",K8/E8)</x:f>
-        <x:v>-0.27939911263320555</x:v>
+        <x:v>-0.2944420119242141</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="43" customHeight="1">
@@ -8662,23 +8662,23 @@
       </x:c>
       <x:c r="H9" s="28" t="n">
         <x:f>MEDIAN('Прогоны'!H25:H27)</x:f>
-        <x:v>3.4994288700000005</x:v>
+        <x:v>3.4032798400000006</x:v>
       </x:c>
       <x:c r="I9" s="28" t="n">
         <x:f>MIN('Прогоны'!H25:H27)</x:f>
-        <x:v>3.3789251000000005</x:v>
+        <x:v>3.3994437</x:v>
       </x:c>
       <x:c r="J9" s="28" t="n">
         <x:f>MAX('Прогоны'!H25:H27)</x:f>
-        <x:v>3.8846642399999993</x:v>
+        <x:v>3.6228520200000007</x:v>
       </x:c>
       <x:c r="K9" s="28" t="n">
         <x:f>H9-E9</x:f>
-        <x:v>-14.03283563</x:v>
+        <x:v>-14.12898466</x:v>
       </x:c>
       <x:c r="L9" s="44" t="n">
         <x:f>IF(E9=0,"",K9/E9)</x:f>
-        <x:v>-0.8004006344987551</x:v>
+        <x:v>-0.8058847537920729</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43" customHeight="1">
@@ -8708,23 +8708,23 @@
       </x:c>
       <x:c r="H10" s="21" t="n">
         <x:f>MEDIAN('Прогоны'!I25:I27)</x:f>
-        <x:v>67.5</x:v>
+        <x:v>86.5</x:v>
       </x:c>
       <x:c r="I10" s="21" t="n">
         <x:f>MIN('Прогоны'!I25:I27)</x:f>
-        <x:v>48</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="J10" s="21" t="n">
         <x:f>MAX('Прогоны'!I25:I27)</x:f>
-        <x:v>108.5</x:v>
+        <x:v>89.00000000000045</x:v>
       </x:c>
       <x:c r="K10" s="21" t="n">
         <x:f>H10-E10</x:f>
-        <x:v>-401.3217999999997</x:v>
+        <x:v>-382.3217999999997</x:v>
       </x:c>
       <x:c r="L10" s="43" t="n">
         <x:f>IF(E10=0,"",K10/E10)</x:f>
-        <x:v>-0.8560220535819792</x:v>
+        <x:v>-0.8154949279235734</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="43" customHeight="1">
@@ -8799,23 +8799,23 @@
       </x:c>
       <x:c r="H12" s="29" t="n">
         <x:f>MEDIAN('Прогоны'!K25:K27)</x:f>
-        <x:v>6.645368347654583</x:v>
+        <x:v>6.884520489319496</x:v>
       </x:c>
       <x:c r="I12" s="29" t="n">
         <x:f>MIN('Прогоны'!K25:K27)</x:f>
-        <x:v>6.585331357014422</x:v>
+        <x:v>6.865107549117331</x:v>
       </x:c>
       <x:c r="J12" s="29" t="n">
         <x:f>MAX('Прогоны'!K25:K27)</x:f>
-        <x:v>6.651752823737132</x:v>
+        <x:v>7.018905840942512</x:v>
       </x:c>
       <x:c r="K12" s="29" t="n">
         <x:f>H12-E12</x:f>
-        <x:v>-6.5443625345054555</x:v>
+        <x:v>-6.305210392840542</x:v>
       </x:c>
       <x:c r="L12" s="43" t="n">
         <x:f>IF(E12=0,"",K12/E12)</x:f>
-        <x:v>-0.49617104344085805</x:v>
+        <x:v>-0.4780393511567962</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="43" customHeight="1">
@@ -8845,23 +8845,23 @@
       </x:c>
       <x:c r="H13" s="20" t="n">
         <x:f>MEDIAN('Прогоны'!L25:L27)</x:f>
-        <x:v>998</x:v>
+        <x:v>1116</x:v>
       </x:c>
       <x:c r="I13" s="20" t="n">
         <x:f>MIN('Прогоны'!L25:L27)</x:f>
-        <x:v>988</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J13" s="20" t="n">
         <x:f>MAX('Прогоны'!L25:L27)</x:f>
-        <x:v>1096</x:v>
+        <x:v>1142</x:v>
       </x:c>
       <x:c r="K13" s="20" t="n">
         <x:f>H13-E13</x:f>
-        <x:v>-72</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="L13" s="44" t="n">
         <x:f>IF(E13=0,"",K13/E13)</x:f>
-        <x:v>-0.06728971962616823</x:v>
+        <x:v>0.04299065420560748</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="43" customHeight="1">
@@ -8891,23 +8891,23 @@
       </x:c>
       <x:c r="H14" s="21" t="n">
         <x:f>MEDIAN('Прогоны'!M25:M27)</x:f>
-        <x:v>1292654</x:v>
+        <x:v>1292830</x:v>
       </x:c>
       <x:c r="I14" s="21" t="n">
         <x:f>MIN('Прогоны'!M25:M27)</x:f>
-        <x:v>1292278</x:v>
+        <x:v>1292762</x:v>
       </x:c>
       <x:c r="J14" s="21" t="n">
         <x:f>MAX('Прогоны'!M25:M27)</x:f>
-        <x:v>1292834</x:v>
+        <x:v>1293053</x:v>
       </x:c>
       <x:c r="K14" s="21" t="n">
         <x:f>H14-E14</x:f>
-        <x:v>-12813282</x:v>
+        <x:v>-12813106</x:v>
       </x:c>
       <x:c r="L14" s="43" t="n">
         <x:f>IF(E14=0,"",K14/E14)</x:f>
-        <x:v>-0.9083609907205024</x:v>
+        <x:v>-0.9083485137037344</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="43" customHeight="1">
@@ -8937,23 +8937,23 @@
       </x:c>
       <x:c r="H15" s="20" t="n">
         <x:f>MEDIAN('Прогоны'!N25:N27)</x:f>
-        <x:v>661993</x:v>
+        <x:v>661989</x:v>
       </x:c>
       <x:c r="I15" s="20" t="n">
         <x:f>MIN('Прогоны'!N25:N27)</x:f>
-        <x:v>661681</x:v>
+        <x:v>661989</x:v>
       </x:c>
       <x:c r="J15" s="20" t="n">
         <x:f>MAX('Прогоны'!N25:N27)</x:f>
-        <x:v>662121</x:v>
+        <x:v>661992</x:v>
       </x:c>
       <x:c r="K15" s="20" t="n">
         <x:f>H15-E15</x:f>
-        <x:v>-10246657</x:v>
+        <x:v>-10246661</x:v>
       </x:c>
       <x:c r="L15" s="44" t="n">
         <x:f>IF(E15=0,"",K15/E15)</x:f>
-        <x:v>-0.9393148556420822</x:v>
+        <x:v>-0.9393152223235689</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="43" customHeight="1">
@@ -8983,23 +8983,23 @@
       </x:c>
       <x:c r="H16" s="21" t="n">
         <x:f>MEDIAN('Прогоны'!O25:O27)</x:f>
-        <x:v>305315</x:v>
+        <x:v>305223</x:v>
       </x:c>
       <x:c r="I16" s="21" t="n">
         <x:f>MIN('Прогоны'!O25:O27)</x:f>
-        <x:v>305232</x:v>
+        <x:v>305222</x:v>
       </x:c>
       <x:c r="J16" s="21" t="n">
         <x:f>MAX('Прогоны'!O25:O27)</x:f>
-        <x:v>305500</x:v>
+        <x:v>305254</x:v>
       </x:c>
       <x:c r="K16" s="21" t="n">
         <x:f>H16-E16</x:f>
-        <x:v>-2109830</x:v>
+        <x:v>-2109922</x:v>
       </x:c>
       <x:c r="L16" s="43" t="n">
         <x:f>IF(E16=0,"",K16/E16)</x:f>
-        <x:v>-0.8735831596032536</x:v>
+        <x:v>-0.8736212525541944</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="43" customHeight="1">
@@ -9075,23 +9075,23 @@
       </x:c>
       <x:c r="H18" s="21" t="n">
         <x:f>MEDIAN('Прогоны'!Q25:Q27)</x:f>
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="I18" s="21" t="n">
         <x:f>MIN('Прогоны'!Q25:Q27)</x:f>
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="J18" s="21" t="n">
         <x:f>MAX('Прогоны'!Q25:Q27)</x:f>
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="K18" s="21" t="n">
         <x:f>H18-E18</x:f>
-        <x:v>-114845</x:v>
+        <x:v>-114632</x:v>
       </x:c>
       <x:c r="L18" s="43" t="n">
         <x:f>IF(E18=0,"",K18/E18)</x:f>
-        <x:v>-0.7900403120399543</x:v>
+        <x:v>-0.7885750450586795</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="43" customHeight="1">
@@ -9167,23 +9167,23 @@
       </x:c>
       <x:c r="H20" s="37" t="n">
         <x:f>MEDIAN('Прогоны'!F28:F30)</x:f>
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I20" s="37" t="n">
         <x:f>MIN('Прогоны'!F28:F30)</x:f>
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="J20" s="37" t="n">
         <x:f>MAX('Прогоны'!F28:F30)</x:f>
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="K20" s="37" t="n">
         <x:f>H20-E20</x:f>
-        <x:v>15.999999999999993</x:v>
+        <x:v>13.999999999999993</x:v>
       </x:c>
       <x:c r="L20" s="45" t="n">
         <x:f>IF(E20=0,"",K20/E20)</x:f>
-        <x:v>0.28571428571428553</x:v>
+        <x:v>0.24999999999999983</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="43" customHeight="1">
@@ -9213,23 +9213,23 @@
       </x:c>
       <x:c r="H21" s="28" t="n">
         <x:f>MEDIAN('Прогоны'!G28:G30)</x:f>
-        <x:v>2.12293024</x:v>
+        <x:v>2.2277842</x:v>
       </x:c>
       <x:c r="I21" s="28" t="n">
         <x:f>MIN('Прогоны'!G28:G30)</x:f>
-        <x:v>2.0799576400000004</x:v>
+        <x:v>2.2196166</x:v>
       </x:c>
       <x:c r="J21" s="28" t="n">
         <x:f>MAX('Прогоны'!G28:G30)</x:f>
-        <x:v>2.2130944000000006</x:v>
+        <x:v>2.3140885999999994</x:v>
       </x:c>
       <x:c r="K21" s="28" t="n">
         <x:f>H21-E21</x:f>
-        <x:v>-1.8581468399999994</x:v>
+        <x:v>-1.7532928799999996</x:v>
       </x:c>
       <x:c r="L21" s="44" t="n">
         <x:f>IF(E21=0,"",K21/E21)</x:f>
-        <x:v>-0.4667447534072864</x:v>
+        <x:v>-0.4404066650224215</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="43" customHeight="1">
@@ -9259,23 +9259,23 @@
       </x:c>
       <x:c r="H22" s="29" t="n">
         <x:f>MEDIAN('Прогоны'!H28:H30)</x:f>
-        <x:v>2.4379597800000004</x:v>
+        <x:v>2.5601073999999997</x:v>
       </x:c>
       <x:c r="I22" s="29" t="n">
         <x:f>MIN('Прогоны'!H28:H30)</x:f>
-        <x:v>2.3842510800000003</x:v>
+        <x:v>2.5481597000000002</x:v>
       </x:c>
       <x:c r="J22" s="29" t="n">
         <x:f>MAX('Прогоны'!H28:H30)</x:f>
-        <x:v>2.5420123</x:v>
+        <x:v>2.6429846999999995</x:v>
       </x:c>
       <x:c r="K22" s="29" t="n">
         <x:f>H22-E22</x:f>
-        <x:v>-3.8714058199999983</x:v>
+        <x:v>-3.749258199999999</x:v>
       </x:c>
       <x:c r="L22" s="43" t="n">
         <x:f>IF(E22=0,"",K22/E22)</x:f>
-        <x:v>-0.6135966855368151</x:v>
+        <x:v>-0.5942369546630805</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="43" customHeight="1">
@@ -9351,7 +9351,7 @@
       </x:c>
       <x:c r="H24" s="33" t="n">
         <x:f>MEDIAN('Прогоны'!J28:J30)</x:f>
-        <x:v>0.010211079982200109</x:v>
+        <x:v>0.01063298715477277</x:v>
       </x:c>
       <x:c r="I24" s="33" t="n">
         <x:f>MIN('Прогоны'!J28:J30)</x:f>
@@ -9363,11 +9363,11 @@
       </x:c>
       <x:c r="K24" s="33" t="n">
         <x:f>H24-E24</x:f>
-        <x:v>-0.0007249511502923616</x:v>
+        <x:v>-0.00030304397771970144</x:v>
       </x:c>
       <x:c r="L24" s="43" t="n">
         <x:f>IF(E24=0,"",K24/E24)</x:f>
-        <x:v>-0.0662901505591394</x:v>
+        <x:v>-0.027710599398287704</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="43" customHeight="1">
@@ -9397,23 +9397,23 @@
       </x:c>
       <x:c r="H25" s="28" t="n">
         <x:f>MEDIAN('Прогоны'!K28:K30)</x:f>
-        <x:v>3.136093933675804</x:v>
+        <x:v>3.23618332667054</x:v>
       </x:c>
       <x:c r="I25" s="28" t="n">
         <x:f>MIN('Прогоны'!K28:K30)</x:f>
-        <x:v>3.061819917493851</x:v>
+        <x:v>3.2109748204783974</x:v>
       </x:c>
       <x:c r="J25" s="28" t="n">
         <x:f>MAX('Прогоны'!K28:K30)</x:f>
-        <x:v>3.519720853646605</x:v>
+        <x:v>3.3636949319726734</x:v>
       </x:c>
       <x:c r="K25" s="28" t="n">
         <x:f>H25-E25</x:f>
-        <x:v>-3.5341645053036475</x:v>
+        <x:v>-3.4340751123089115</x:v>
       </x:c>
       <x:c r="L25" s="44" t="n">
         <x:f>IF(E25=0,"",K25/E25)</x:f>
-        <x:v>-0.5298392165213278</x:v>
+        <x:v>-0.5148338919285299</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="43" customHeight="1">
@@ -9443,23 +9443,23 @@
       </x:c>
       <x:c r="H26" s="21" t="n">
         <x:f>MEDIAN('Прогоны'!L28:L30)</x:f>
-        <x:v>1041</x:v>
+        <x:v>1144</x:v>
       </x:c>
       <x:c r="I26" s="21" t="n">
         <x:f>MIN('Прогоны'!L28:L30)</x:f>
-        <x:v>1040</x:v>
+        <x:v>1103</x:v>
       </x:c>
       <x:c r="J26" s="21" t="n">
         <x:f>MAX('Прогоны'!L28:L30)</x:f>
-        <x:v>1164</x:v>
+        <x:v>1153</x:v>
       </x:c>
       <x:c r="K26" s="21" t="n">
         <x:f>H26-E26</x:f>
-        <x:v>-87</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="L26" s="43" t="n">
         <x:f>IF(E26=0,"",K26/E26)</x:f>
-        <x:v>-0.07712765957446809</x:v>
+        <x:v>0.014184397163120567</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="43" customHeight="1">
@@ -9489,23 +9489,23 @@
       </x:c>
       <x:c r="H27" s="20" t="n">
         <x:f>MEDIAN('Прогоны'!M28:M30)</x:f>
-        <x:v>2367913</x:v>
+        <x:v>2368338</x:v>
       </x:c>
       <x:c r="I27" s="20" t="n">
         <x:f>MIN('Прогоны'!M28:M30)</x:f>
-        <x:v>2367837</x:v>
+        <x:v>2368219</x:v>
       </x:c>
       <x:c r="J27" s="20" t="n">
         <x:f>MAX('Прогоны'!M28:M30)</x:f>
-        <x:v>2367974</x:v>
+        <x:v>2368382</x:v>
       </x:c>
       <x:c r="K27" s="20" t="n">
         <x:f>H27-E27</x:f>
-        <x:v>-11797747</x:v>
+        <x:v>-11797322</x:v>
       </x:c>
       <x:c r="L27" s="44" t="n">
         <x:f>IF(E27=0,"",K27/E27)</x:f>
-        <x:v>-0.8328413219009916</x:v>
+        <x:v>-0.8328113197690754</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="43" customHeight="1">
@@ -9535,23 +9535,23 @@
       </x:c>
       <x:c r="H28" s="21" t="n">
         <x:f>MEDIAN('Прогоны'!N28:N30)</x:f>
-        <x:v>1737303</x:v>
+        <x:v>1737435</x:v>
       </x:c>
       <x:c r="I28" s="21" t="n">
         <x:f>MIN('Прогоны'!N28:N30)</x:f>
-        <x:v>1737302</x:v>
+        <x:v>1737305</x:v>
       </x:c>
       <x:c r="J28" s="21" t="n">
         <x:f>MAX('Прогоны'!N28:N30)</x:f>
-        <x:v>1737435</x:v>
+        <x:v>1737436</x:v>
       </x:c>
       <x:c r="K28" s="21" t="n">
         <x:f>H28-E28</x:f>
-        <x:v>-9218276</x:v>
+        <x:v>-9218144</x:v>
       </x:c>
       <x:c r="L28" s="43" t="n">
         <x:f>IF(E28=0,"",K28/E28)</x:f>
-        <x:v>-0.8414229864071995</x:v>
+        <x:v>-0.8414109377514415</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="43" customHeight="1">
@@ -9581,23 +9581,23 @@
       </x:c>
       <x:c r="H29" s="20" t="n">
         <x:f>MEDIAN('Прогоны'!O28:O30)</x:f>
-        <x:v>305211</x:v>
+        <x:v>305267</x:v>
       </x:c>
       <x:c r="I29" s="20" t="n">
         <x:f>MIN('Прогоны'!O28:O30)</x:f>
-        <x:v>305209</x:v>
+        <x:v>305213</x:v>
       </x:c>
       <x:c r="J29" s="20" t="n">
         <x:f>MAX('Прогоны'!O28:O30)</x:f>
-        <x:v>305241</x:v>
+        <x:v>305356</x:v>
       </x:c>
       <x:c r="K29" s="20" t="n">
         <x:f>H29-E29</x:f>
-        <x:v>-2109950</x:v>
+        <x:v>-2109894</x:v>
       </x:c>
       <x:c r="L29" s="44" t="n">
         <x:f>IF(E29=0,"",K29/E29)</x:f>
-        <x:v>-0.8736270584031458</x:v>
+        <x:v>-0.8736038715431393</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="43" customHeight="1">
@@ -9673,23 +9673,23 @@
       </x:c>
       <x:c r="H31" s="20" t="n">
         <x:f>MEDIAN('Прогоны'!Q28:Q30)</x:f>
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="I31" s="20" t="n">
         <x:f>MIN('Прогоны'!Q28:Q30)</x:f>
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="J31" s="20" t="n">
         <x:f>MAX('Прогоны'!Q28:Q30)</x:f>
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="K31" s="20" t="n">
         <x:f>H31-E31</x:f>
-        <x:v>-114848</x:v>
+        <x:v>-114635</x:v>
       </x:c>
       <x:c r="L31" s="44" t="n">
         <x:f>IF(E31=0,"",K31/E31)</x:f>
-        <x:v>-0.7900446450068447</x:v>
+        <x:v>-0.7885794082644856</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="43" customHeight="1">
@@ -13404,43 +13404,43 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E25" s="24" t="n">
-        <x:v>46302.75725248842</x:v>
+        <x:v>46302.84509113426</x:v>
       </x:c>
       <x:c r="F25" s="20" t="n">
         <x:v>79</x:v>
       </x:c>
       <x:c r="G25" s="28" t="n">
-        <x:v>3.3789251</x:v>
+        <x:v>3.3994437</x:v>
       </x:c>
       <x:c r="H25" s="28" t="n">
-        <x:v>3.3789251000000005</x:v>
+        <x:v>3.3994437</x:v>
       </x:c>
       <x:c r="I25" s="20" t="n">
-        <x:v>67.5</x:v>
+        <x:v>89.00000000000045</x:v>
       </x:c>
       <x:c r="J25" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K25" s="28" t="n">
-        <x:v>6.645368347654583</x:v>
+        <x:v>6.884520489319496</x:v>
       </x:c>
       <x:c r="L25" s="20" t="n">
-        <x:v>1096</x:v>
+        <x:v>1142</x:v>
       </x:c>
       <x:c r="M25" s="20" t="n">
-        <x:v>1292834</x:v>
+        <x:v>1293053</x:v>
       </x:c>
       <x:c r="N25" s="20" t="n">
-        <x:v>661993</x:v>
+        <x:v>661989</x:v>
       </x:c>
       <x:c r="O25" s="20" t="n">
-        <x:v>305500</x:v>
+        <x:v>305254</x:v>
       </x:c>
       <x:c r="P25" s="20" t="n">
         <x:v>220618</x:v>
       </x:c>
       <x:c r="Q25" s="20" t="n">
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="R25" s="20" t="n">
         <x:v>70</x:v>
@@ -13463,43 +13463,43 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E26" s="25" t="n">
-        <x:v>46302.757514826386</x:v>
+        <x:v>46302.84536259259</x:v>
       </x:c>
       <x:c r="F26" s="21" t="n">
-        <x:v>75</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="G26" s="29" t="n">
-        <x:v>3.4758397099999994</x:v>
+        <x:v>3.4032798400000006</x:v>
       </x:c>
       <x:c r="H26" s="29" t="n">
-        <x:v>3.8846642399999993</x:v>
+        <x:v>3.4032798400000006</x:v>
       </x:c>
       <x:c r="I26" s="21" t="n">
-        <x:v>108.5</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="J26" s="33" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K26" s="29" t="n">
-        <x:v>6.585331357014422</x:v>
+        <x:v>6.865107549117331</x:v>
       </x:c>
       <x:c r="L26" s="21" t="n">
-        <x:v>988</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="M26" s="21" t="n">
-        <x:v>1292278</x:v>
+        <x:v>1292762</x:v>
       </x:c>
       <x:c r="N26" s="21" t="n">
-        <x:v>661681</x:v>
+        <x:v>661989</x:v>
       </x:c>
       <x:c r="O26" s="21" t="n">
-        <x:v>305315</x:v>
+        <x:v>305223</x:v>
       </x:c>
       <x:c r="P26" s="21" t="n">
         <x:v>220618</x:v>
       </x:c>
       <x:c r="Q26" s="21" t="n">
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="R26" s="21" t="n">
         <x:v>70</x:v>
@@ -13522,43 +13522,43 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E27" s="24" t="n">
-        <x:v>46302.75778034722</x:v>
+        <x:v>46302.8456296875</x:v>
       </x:c>
       <x:c r="F27" s="20" t="n">
-        <x:v>78</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="G27" s="28" t="n">
-        <x:v>3.49942887</x:v>
+        <x:v>3.6228520200000003</x:v>
       </x:c>
       <x:c r="H27" s="28" t="n">
-        <x:v>3.4994288700000005</x:v>
+        <x:v>3.6228520200000007</x:v>
       </x:c>
       <x:c r="I27" s="20" t="n">
-        <x:v>48</x:v>
+        <x:v>86.5</x:v>
       </x:c>
       <x:c r="J27" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K27" s="28" t="n">
-        <x:v>6.651752823737132</x:v>
+        <x:v>7.018905840942512</x:v>
       </x:c>
       <x:c r="L27" s="20" t="n">
-        <x:v>998</x:v>
+        <x:v>1116</x:v>
       </x:c>
       <x:c r="M27" s="20" t="n">
-        <x:v>1292654</x:v>
+        <x:v>1292830</x:v>
       </x:c>
       <x:c r="N27" s="20" t="n">
-        <x:v>662121</x:v>
+        <x:v>661992</x:v>
       </x:c>
       <x:c r="O27" s="20" t="n">
-        <x:v>305232</x:v>
+        <x:v>305222</x:v>
       </x:c>
       <x:c r="P27" s="20" t="n">
         <x:v>220618</x:v>
       </x:c>
       <x:c r="Q27" s="20" t="n">
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="R27" s="20" t="n">
         <x:v>70</x:v>
@@ -13581,43 +13581,43 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E28" s="25" t="n">
-        <x:v>46302.75805960648</x:v>
+        <x:v>46302.845899189815</x:v>
       </x:c>
       <x:c r="F28" s="21" t="n">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="G28" s="29" t="n">
-        <x:v>2.12293024</x:v>
+        <x:v>2.2277842</x:v>
       </x:c>
       <x:c r="H28" s="29" t="n">
-        <x:v>2.4379597800000004</x:v>
+        <x:v>2.5601073999999997</x:v>
       </x:c>
       <x:c r="I28" s="21" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J28" s="33" t="n">
-        <x:v>0.010211079982200109</x:v>
+        <x:v>0.01063298715477277</x:v>
       </x:c>
       <x:c r="K28" s="29" t="n">
-        <x:v>3.061819917493851</x:v>
+        <x:v>3.2109748204783974</x:v>
       </x:c>
       <x:c r="L28" s="21" t="n">
-        <x:v>1040</x:v>
+        <x:v>1153</x:v>
       </x:c>
       <x:c r="M28" s="21" t="n">
-        <x:v>2367913</x:v>
+        <x:v>2368338</x:v>
       </x:c>
       <x:c r="N28" s="21" t="n">
-        <x:v>1737302</x:v>
+        <x:v>1737435</x:v>
       </x:c>
       <x:c r="O28" s="21" t="n">
-        <x:v>305241</x:v>
+        <x:v>305267</x:v>
       </x:c>
       <x:c r="P28" s="21" t="n">
         <x:v>220618</x:v>
       </x:c>
       <x:c r="Q28" s="21" t="n">
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="R28" s="21" t="n">
         <x:v>80</x:v>
@@ -13640,43 +13640,43 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E29" s="24" t="n">
-        <x:v>46302.75833747685</x:v>
+        <x:v>46302.84618689815</x:v>
       </x:c>
       <x:c r="F29" s="20" t="n">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="G29" s="28" t="n">
-        <x:v>2.2130944000000006</x:v>
+        <x:v>2.3140885999999994</x:v>
       </x:c>
       <x:c r="H29" s="28" t="n">
-        <x:v>2.5420123</x:v>
+        <x:v>2.6429846999999995</x:v>
       </x:c>
       <x:c r="I29" s="20" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J29" s="32" t="n">
-        <x:v>0.01063298715477277</x:v>
+        <x:v>0.010211079982200109</x:v>
       </x:c>
       <x:c r="K29" s="28" t="n">
-        <x:v>3.519720853646605</x:v>
+        <x:v>3.3636949319726734</x:v>
       </x:c>
       <x:c r="L29" s="20" t="n">
-        <x:v>1164</x:v>
+        <x:v>1103</x:v>
       </x:c>
       <x:c r="M29" s="20" t="n">
-        <x:v>2367974</x:v>
+        <x:v>2368382</x:v>
       </x:c>
       <x:c r="N29" s="20" t="n">
-        <x:v>1737435</x:v>
+        <x:v>1737305</x:v>
       </x:c>
       <x:c r="O29" s="20" t="n">
-        <x:v>305209</x:v>
+        <x:v>305356</x:v>
       </x:c>
       <x:c r="P29" s="20" t="n">
         <x:v>220618</x:v>
       </x:c>
       <x:c r="Q29" s="20" t="n">
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="R29" s="20" t="n">
         <x:v>80</x:v>
@@ -13699,43 +13699,43 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E30" s="25" t="n">
-        <x:v>46302.758625138886</x:v>
+        <x:v>46302.84646997685</x:v>
       </x:c>
       <x:c r="F30" s="21" t="n">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="G30" s="29" t="n">
-        <x:v>2.0799576400000004</x:v>
+        <x:v>2.2196166</x:v>
       </x:c>
       <x:c r="H30" s="29" t="n">
-        <x:v>2.3842510800000003</x:v>
+        <x:v>2.5481597000000002</x:v>
       </x:c>
       <x:c r="I30" s="21" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J30" s="33" t="n">
-        <x:v>0.010211079982200109</x:v>
+        <x:v>0.01063298715477277</x:v>
       </x:c>
       <x:c r="K30" s="29" t="n">
-        <x:v>3.136093933675804</x:v>
+        <x:v>3.23618332667054</x:v>
       </x:c>
       <x:c r="L30" s="21" t="n">
-        <x:v>1041</x:v>
+        <x:v>1144</x:v>
       </x:c>
       <x:c r="M30" s="21" t="n">
-        <x:v>2367837</x:v>
+        <x:v>2368219</x:v>
       </x:c>
       <x:c r="N30" s="21" t="n">
-        <x:v>1737303</x:v>
+        <x:v>1737436</x:v>
       </x:c>
       <x:c r="O30" s="21" t="n">
-        <x:v>305211</x:v>
+        <x:v>305213</x:v>
       </x:c>
       <x:c r="P30" s="21" t="n">
         <x:v>220618</x:v>
       </x:c>
       <x:c r="Q30" s="21" t="n">
-        <x:v>30521</x:v>
+        <x:v>30734</x:v>
       </x:c>
       <x:c r="R30" s="21" t="n">
         <x:v>80</x:v>

</xml_diff>